<commit_message>
Update 十三里屋 inventory sheet with confirmed quantities
- ヤキスイ: 単位パック・数量42（単価は1パック=1kg換算の630円）
- あんこ: 14kg（単価677円/kg）
- ハナ雛形から引き継いだ番号重複(23)と不要な式を修正
- 単価・数量が未確定の品目は行だけ残して空欄
合計 347,962円。Google スプレッドシート版をDriveの十三里屋フォルダにアップロード。

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019UT53ngJ9KbuULNgo6kMHm
</commit_message>
<xml_diff>
--- a/棚卸表/棚卸表_さわら十三里屋_20260831.xlsx
+++ b/棚卸表/棚卸表_さわら十三里屋_20260831.xlsx
@@ -1608,12 +1608,14 @@
       <c r="E16" s="41" t="n"/>
       <c r="F16" s="42" t="n"/>
       <c r="G16" s="58" t="n">
-        <v>6300</v>
-      </c>
-      <c r="H16" s="56" t="n"/>
+        <v>630</v>
+      </c>
+      <c r="H16" s="56" t="n">
+        <v>42</v>
+      </c>
       <c r="I16" s="57" t="inlineStr">
         <is>
-          <t>C/S</t>
+          <t>パック</t>
         </is>
       </c>
       <c r="J16" s="58">
@@ -2329,7 +2331,7 @@
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="3" t="n"/>
       <c r="B28" s="8" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C28" s="54" t="inlineStr">
         <is>
@@ -3033,21 +3035,21 @@
       </c>
       <c r="C41" s="54" t="inlineStr">
         <is>
-          <t>あんこ　2kg</t>
+          <t>あんこ</t>
         </is>
       </c>
       <c r="D41" s="41" t="n"/>
       <c r="E41" s="41" t="n"/>
       <c r="F41" s="42" t="n"/>
       <c r="G41" s="58" t="n">
-        <v>1354</v>
+        <v>677</v>
       </c>
       <c r="H41" s="56" t="n">
         <v>14</v>
       </c>
       <c r="I41" s="57" t="inlineStr">
         <is>
-          <t>2kg</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="J41" s="58">
@@ -3269,10 +3271,7 @@
         <f>Q45*R45</f>
         <v/>
       </c>
-      <c r="U45" s="61">
-        <f>SUM(T48:T56)</f>
-        <v/>
-      </c>
+      <c r="U45" s="61" t="n"/>
       <c r="V45" s="3" t="n"/>
       <c r="W45" s="3" t="n"/>
       <c r="X45" s="3" t="n"/>

</xml_diff>